<commit_message>
add number of channel cols
</commit_message>
<xml_diff>
--- a/auto_watch.xlsx
+++ b/auto_watch.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,20 +428,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>channel_count</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>comment</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>like</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>search</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>like_comment_count</t>
         </is>
@@ -453,22 +458,25 @@
           <t>a;b;c;d;e;f;g;h;j</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>false;This took most of the day and required multiple approaches and many failed attempts, but I did eventually get it installed via the very cool stable-diffusion-webui project. Excited, I immediately start generating a picture of a litter of kittens cuddling and sleeping together, because what else could I possibly generate?;Suddenly the microwave timer goes off. Food is done I guess. I didn't realize my partner was heating up dinner already, it is a little early for that. Microwave's tone sounds a bit off too, I hope it isn't broken or something.;false;This took most of the day and required multiple approaches and many failed attempts, but I did eventually get it installed via the very cool stable-diffusion-webui project. Excited, I immediately start generating a picture of a litter of kittens cuddling and sleeping together, because what else could I possibly generate?</t>
-        </is>
+      <c r="B2" t="n">
+        <v>9</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>false;false;false;false;false</t>
+          <t>false;false;false;false;Suddenly the microwave timer goes off. Food is done I guess. I didn't realize my partner was heating up dinner already, it is a little early for that. Microwave's tone sounds a bit off too, I hope it isn't broken or something.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>def;false;123;123;123</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+          <t>false;false;false;true;false</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>false;def;def;false;def</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -478,22 +486,25 @@
           <t>a;b;c;d;e;f;g;h;j</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>But more importantly, I now have a cute (if a little creepy) picture of kittens!;false;But more importantly, I now have a cute (if a little creepy) picture of kittens!;false;This took most of the day and required multiple approaches and many failed attempts, but I did eventually get it installed via the very cool stable-diffusion-webui project. Excited, I immediately start generating a picture of a litter of kittens cuddling and sleeping together, because what else could I possibly generate?</t>
-        </is>
+      <c r="B3" t="n">
+        <v>9</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>false;But more importantly, I now have a cute (if a little creepy) picture of kittens!;false;Suddenly the microwave timer goes off. Food is done I guess. I didn't realize my partner was heating up dinner already, it is a little early for that. Microwave's tone sounds a bit off too, I hope it isn't broken or something.;Suddenly the microwave timer goes off. Food is done I guess. I didn't realize my partner was heating up dinner already, it is a little early for that. Microwave's tone sounds a bit off too, I hope it isn't broken or something.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>false;false;false;false;false</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>def;false;false;123;def</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>123;false;def;123;false</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>